<commit_message>
added variance and some hackishness, to not much purpose probably
</commit_message>
<xml_diff>
--- a/src/templates/report.xlsx
+++ b/src/templates/report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Luke\Computer Science\repos\cpf-concours\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA65B354-367D-4B3E-8A79-70AB32DC8C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C94C3B0-5AF4-4538-9013-0113F00A4514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="contestants" sheetId="23" r:id="rId1"/>
@@ -18,14 +18,15 @@
     <sheet name="judges" sheetId="1" r:id="rId3"/>
     <sheet name="judges_adjust" sheetId="11" r:id="rId4"/>
     <sheet name="categories" sheetId="16" r:id="rId5"/>
-    <sheet name="formats" sheetId="17" r:id="rId6"/>
-    <sheet name="grades" sheetId="22" r:id="rId7"/>
-    <sheet name="levels" sheetId="21" r:id="rId8"/>
-    <sheet name="durations" sheetId="20" r:id="rId9"/>
-    <sheet name="durations_adjust" sheetId="25" r:id="rId10"/>
-    <sheet name="schools_given" sheetId="19" r:id="rId11"/>
-    <sheet name="schools_received" sheetId="18" r:id="rId12"/>
-    <sheet name="places" sheetId="8" r:id="rId13"/>
+    <sheet name="category_variances" sheetId="26" r:id="rId6"/>
+    <sheet name="formats" sheetId="17" r:id="rId7"/>
+    <sheet name="grades" sheetId="22" r:id="rId8"/>
+    <sheet name="levels" sheetId="21" r:id="rId9"/>
+    <sheet name="durations" sheetId="20" r:id="rId10"/>
+    <sheet name="durations_adjust" sheetId="25" r:id="rId11"/>
+    <sheet name="schools_given" sheetId="19" r:id="rId12"/>
+    <sheet name="schools_received" sheetId="18" r:id="rId13"/>
+    <sheet name="places" sheetId="8" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="34">
   <si>
     <t>Judge</t>
   </si>
@@ -225,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -234,7 +235,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,6 +587,72 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{653CBE1A-FE09-45DA-8160-361132CBEAED}">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E1ABD5-ADB2-4DF0-BFBA-D2844F79AC2C}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -652,7 +718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9428BBEB-AE09-4206-8D75-ED9A87413722}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -718,7 +784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F08DCBB-D175-4513-8600-35D4C74F475D}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -784,12 +850,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80F715B5-CDA7-4378-A61A-53470693CA9F}">
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="8" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" customWidth="1"/>
     <col min="2" max="11" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1099,6 +1165,72 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA00A54-28E9-497D-9F41-B6E51533DE81}">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38439C5D-7B17-4C5A-8E3A-1DEAF695CFA4}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1164,7 +1296,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{655E84FE-8528-42DB-81A6-BC97A0E9D785}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1230,7 +1362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82842637-9C55-4613-9A3D-5E83244837E9}">
   <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1294,70 +1426,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{653CBE1A-FE09-45DA-8160-361132CBEAED}">
-  <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="22.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>